<commit_message>
Changed the UI of user-side appointment, added more security towards booking
</commit_message>
<xml_diff>
--- a/SG-Confidential.xlsx
+++ b/SG-Confidential.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ron\OneDrive - STI College Las Pinas\Desktop\Capstone2026\Website\Compilation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/863cfc00ecbb8e58/- STI College Las Pinas/Desktop/Capstone2026/Cursor/Website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC3DCE5-2934-4291-B3BE-DC7F083A018F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{BBC3DCE5-2934-4291-B3BE-DC7F083A018F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7DE92A0-55F4-4B0E-863B-C9BA09B5503C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11175" yWindow="1065" windowWidth="17130" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Name and Position " sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="179">
   <si>
     <t>Name</t>
   </si>
@@ -554,12 +554,18 @@
   <si>
     <t>Whole Body w/ BFR &amp; BT</t>
   </si>
+  <si>
+    <t>geraselragudo123@gmail.com</t>
+  </si>
+  <si>
+    <t>loidadeguzman123@gmail.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -639,6 +645,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -657,10 +670,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -685,6 +699,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -693,7 +708,8 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -707,6 +723,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -913,9 +933,10 @@
   <dimension ref="A1:Z1001"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="57.85546875" customWidth="1"/>
-    <col min="3" max="4" width="15.85546875" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="67.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -950,7 +971,7 @@
       <c r="Y1" s="4"/>
       <c r="Z1" s="4"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
@@ -982,7 +1003,7 @@
       <c r="Y2" s="4"/>
       <c r="Z2" s="4"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1014,7 +1035,7 @@
       <c r="Y3" s="4"/>
       <c r="Z3" s="4"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -1046,14 +1067,16 @@
       <c r="Y4" s="4"/>
       <c r="Z4" s="4"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="14" t="s">
+        <v>177</v>
+      </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -1078,7 +1101,7 @@
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -1110,14 +1133,16 @@
       <c r="Y6" s="4"/>
       <c r="Z6" s="4"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="14" t="s">
+        <v>178</v>
+      </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -1142,7 +1167,7 @@
       <c r="Y7" s="4"/>
       <c r="Z7" s="4"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
@@ -1174,7 +1199,7 @@
       <c r="Y8" s="4"/>
       <c r="Z8" s="4"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1234,7 +1259,7 @@
       <c r="Y10" s="4"/>
       <c r="Z10" s="4"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1262,7 +1287,7 @@
       <c r="Y11" s="4"/>
       <c r="Z11" s="4"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1290,7 +1315,7 @@
       <c r="Y12" s="4"/>
       <c r="Z12" s="4"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1318,7 +1343,7 @@
       <c r="Y13" s="4"/>
       <c r="Z13" s="4"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1346,7 +1371,7 @@
       <c r="Y14" s="4"/>
       <c r="Z14" s="4"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1374,7 +1399,7 @@
       <c r="Y15" s="4"/>
       <c r="Z15" s="4"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1402,7 +1427,7 @@
       <c r="Y16" s="4"/>
       <c r="Z16" s="4"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1430,7 +1455,7 @@
       <c r="Y17" s="4"/>
       <c r="Z17" s="4"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1458,7 +1483,7 @@
       <c r="Y18" s="4"/>
       <c r="Z18" s="4"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1486,7 +1511,7 @@
       <c r="Y19" s="4"/>
       <c r="Z19" s="4"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1514,7 +1539,7 @@
       <c r="Y20" s="4"/>
       <c r="Z20" s="4"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1542,7 +1567,7 @@
       <c r="Y21" s="4"/>
       <c r="Z21" s="4"/>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1570,7 +1595,7 @@
       <c r="Y22" s="4"/>
       <c r="Z22" s="4"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1598,7 +1623,7 @@
       <c r="Y23" s="4"/>
       <c r="Z23" s="4"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1626,7 +1651,7 @@
       <c r="Y24" s="4"/>
       <c r="Z24" s="4"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1654,7 +1679,7 @@
       <c r="Y25" s="4"/>
       <c r="Z25" s="4"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1682,7 +1707,7 @@
       <c r="Y26" s="4"/>
       <c r="Z26" s="4"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1710,7 +1735,7 @@
       <c r="Y27" s="4"/>
       <c r="Z27" s="4"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1738,7 +1763,7 @@
       <c r="Y28" s="4"/>
       <c r="Z28" s="4"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1766,7 +1791,7 @@
       <c r="Y29" s="4"/>
       <c r="Z29" s="4"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1794,7 +1819,7 @@
       <c r="Y30" s="4"/>
       <c r="Z30" s="4"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1822,7 +1847,7 @@
       <c r="Y31" s="4"/>
       <c r="Z31" s="4"/>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1850,7 +1875,7 @@
       <c r="Y32" s="4"/>
       <c r="Z32" s="4"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1878,7 +1903,7 @@
       <c r="Y33" s="4"/>
       <c r="Z33" s="4"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1906,7 +1931,7 @@
       <c r="Y34" s="4"/>
       <c r="Z34" s="4"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -1934,7 +1959,7 @@
       <c r="Y35" s="4"/>
       <c r="Z35" s="4"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -28983,6 +29008,10 @@
       <c r="Z1001" s="4"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{671803E6-546F-4EF9-8823-9596F11DC63C}"/>
+    <hyperlink ref="C7" r:id="rId2" xr:uid="{51360B51-5354-49D2-969A-C25FABD81177}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -44115,22 +44144,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="D1" s="16" t="s">
+      <c r="B1" s="16"/>
+      <c r="D1" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="15"/>
-      <c r="G1" s="14" t="s">
+      <c r="E1" s="16"/>
+      <c r="G1" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="J1" s="16" t="s">
+      <c r="H1" s="16"/>
+      <c r="J1" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="K1" s="15"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
@@ -44281,18 +44310,18 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="D10" s="16" t="s">
+      <c r="B10" s="16"/>
+      <c r="D10" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="G10" s="16" t="s">
+      <c r="E10" s="16"/>
+      <c r="G10" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="15"/>
+      <c r="H10" s="16"/>
       <c r="J10" s="9" t="s">
         <v>110</v>
       </c>
@@ -44452,24 +44481,24 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="D19" s="16" t="s">
+      <c r="B19" s="16"/>
+      <c r="D19" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="16"/>
       <c r="G19" s="9" t="s">
         <v>134</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="J19" s="16" t="s">
+      <c r="J19" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="K19" s="15"/>
+      <c r="K19" s="16"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
@@ -44530,10 +44559,10 @@
       <c r="E22" s="10">
         <v>3000</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="H22" s="15"/>
+      <c r="H22" s="16"/>
       <c r="J22" s="9" t="s">
         <v>142</v>
       </c>
@@ -44744,22 +44773,22 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="D32" s="16" t="s">
+      <c r="B32" s="16"/>
+      <c r="D32" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="E32" s="15"/>
+      <c r="E32" s="16"/>
       <c r="G32" s="9" t="s">
         <v>171</v>
       </c>
       <c r="H32" s="10">
         <v>5000</v>
       </c>
-      <c r="J32" s="16"/>
-      <c r="K32" s="15"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="16"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">

</xml_diff>